<commit_message>
walk through limpa quantification, and show where the blood removal backfires
</commit_message>
<xml_diff>
--- a/01_Processing/03_Quantification/c_data/quantification.xlsx
+++ b/01_Processing/03_Quantification/c_data/quantification.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4441" uniqueCount="4045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4474" uniqueCount="4066">
   <si>
     <t>sheet</t>
   </si>
@@ -11927,12 +11927,24 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>foreach</t>
   </si>
   <si>
@@ -11984,6 +11996,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -11996,12 +12020,21 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>limma</t>
   </si>
   <si>
@@ -12026,6 +12059,12 @@
     <t>1.5.0</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -12083,6 +12122,12 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -12140,6 +12185,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -12156,6 +12207,18 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -67301,7 +67364,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -67551,7 +67614,7 @@
         <v>3978</v>
       </c>
       <c r="B23" t="s">
-        <v>3973</v>
+        <v>3979</v>
       </c>
       <c r="C23" t="s">
         <v>3939</v>
@@ -67559,10 +67622,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>3979</v>
+        <v>3980</v>
       </c>
       <c r="B24" t="s">
-        <v>3980</v>
+        <v>3981</v>
       </c>
       <c r="C24" t="s">
         <v>3939</v>
@@ -67570,10 +67633,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>3981</v>
+        <v>3982</v>
       </c>
       <c r="B25" t="s">
-        <v>3982</v>
+        <v>3977</v>
       </c>
       <c r="C25" t="s">
         <v>3939</v>
@@ -67609,7 +67672,7 @@
         <v>3988</v>
       </c>
       <c r="C28" t="s">
-        <v>3936</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -67642,7 +67705,7 @@
         <v>3994</v>
       </c>
       <c r="C31" t="s">
-        <v>3936</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -67694,7 +67757,7 @@
         <v>4003</v>
       </c>
       <c r="B36" t="s">
-        <v>4004</v>
+        <v>3969</v>
       </c>
       <c r="C36" t="s">
         <v>3939</v>
@@ -67702,32 +67765,32 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
+        <v>4004</v>
+      </c>
+      <c r="B37" t="s">
         <v>4005</v>
       </c>
-      <c r="B37" t="s">
-        <v>4006</v>
-      </c>
       <c r="C37" t="s">
-        <v>3939</v>
+        <v>3936</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>4006</v>
+      </c>
+      <c r="B38" t="s">
         <v>4007</v>
       </c>
-      <c r="B38" t="s">
-        <v>4008</v>
-      </c>
       <c r="C38" t="s">
-        <v>3939</v>
+        <v>3936</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>4008</v>
+      </c>
+      <c r="B39" t="s">
         <v>4009</v>
-      </c>
-      <c r="B39" t="s">
-        <v>4010</v>
       </c>
       <c r="C39" t="s">
         <v>3939</v>
@@ -67735,10 +67798,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>4010</v>
+      </c>
+      <c r="B40" t="s">
         <v>4011</v>
-      </c>
-      <c r="B40" t="s">
-        <v>4012</v>
       </c>
       <c r="C40" t="s">
         <v>3939</v>
@@ -67746,10 +67809,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>4012</v>
+      </c>
+      <c r="B41" t="s">
         <v>4013</v>
-      </c>
-      <c r="B41" t="s">
-        <v>4014</v>
       </c>
       <c r="C41" t="s">
         <v>3939</v>
@@ -67757,10 +67820,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>4014</v>
+      </c>
+      <c r="B42" t="s">
         <v>4015</v>
-      </c>
-      <c r="B42" t="s">
-        <v>4016</v>
       </c>
       <c r="C42" t="s">
         <v>3939</v>
@@ -67768,21 +67831,21 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
+        <v>4016</v>
+      </c>
+      <c r="B43" t="s">
         <v>4017</v>
       </c>
-      <c r="B43" t="s">
-        <v>4018</v>
-      </c>
       <c r="C43" t="s">
-        <v>4019</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>4020</v>
+        <v>4018</v>
       </c>
       <c r="B44" t="s">
-        <v>4021</v>
+        <v>4019</v>
       </c>
       <c r="C44" t="s">
         <v>3939</v>
@@ -67790,21 +67853,21 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>4022</v>
+        <v>4020</v>
       </c>
       <c r="B45" t="s">
-        <v>4023</v>
+        <v>4021</v>
       </c>
       <c r="C45" t="s">
-        <v>3936</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>4024</v>
+        <v>4022</v>
       </c>
       <c r="B46" t="s">
-        <v>4025</v>
+        <v>4023</v>
       </c>
       <c r="C46" t="s">
         <v>3939</v>
@@ -67812,10 +67875,10 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>4026</v>
+        <v>4024</v>
       </c>
       <c r="B47" t="s">
-        <v>4027</v>
+        <v>4025</v>
       </c>
       <c r="C47" t="s">
         <v>3939</v>
@@ -67823,10 +67886,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>4028</v>
+        <v>4026</v>
       </c>
       <c r="B48" t="s">
-        <v>4029</v>
+        <v>4027</v>
       </c>
       <c r="C48" t="s">
         <v>3939</v>
@@ -67834,10 +67897,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>4030</v>
+        <v>4028</v>
       </c>
       <c r="B49" t="s">
-        <v>4031</v>
+        <v>4029</v>
       </c>
       <c r="C49" t="s">
         <v>3939</v>
@@ -67845,21 +67908,21 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>4030</v>
+      </c>
+      <c r="B50" t="s">
+        <v>4031</v>
+      </c>
+      <c r="C50" t="s">
         <v>4032</v>
-      </c>
-      <c r="B50" t="s">
-        <v>4033</v>
-      </c>
-      <c r="C50" t="s">
-        <v>3939</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>4033</v>
+      </c>
+      <c r="B51" t="s">
         <v>4034</v>
-      </c>
-      <c r="B51" t="s">
-        <v>4035</v>
       </c>
       <c r="C51" t="s">
         <v>3939</v>
@@ -67867,10 +67930,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>4035</v>
+      </c>
+      <c r="B52" t="s">
         <v>4036</v>
-      </c>
-      <c r="B52" t="s">
-        <v>3967</v>
       </c>
       <c r="C52" t="s">
         <v>3939</v>
@@ -67884,7 +67947,7 @@
         <v>4038</v>
       </c>
       <c r="C53" t="s">
-        <v>3939</v>
+        <v>3936</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -67917,6 +67980,127 @@
         <v>4044</v>
       </c>
       <c r="C56" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>4045</v>
+      </c>
+      <c r="B57" t="s">
+        <v>4046</v>
+      </c>
+      <c r="C57" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>4047</v>
+      </c>
+      <c r="B58" t="s">
+        <v>4048</v>
+      </c>
+      <c r="C58" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>4049</v>
+      </c>
+      <c r="B59" t="s">
+        <v>4050</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>4051</v>
+      </c>
+      <c r="B60" t="s">
+        <v>3967</v>
+      </c>
+      <c r="C60" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>4052</v>
+      </c>
+      <c r="B61" t="s">
+        <v>4053</v>
+      </c>
+      <c r="C61" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>4054</v>
+      </c>
+      <c r="B62" t="s">
+        <v>4055</v>
+      </c>
+      <c r="C62" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>4056</v>
+      </c>
+      <c r="B63" t="s">
+        <v>4057</v>
+      </c>
+      <c r="C63" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>4058</v>
+      </c>
+      <c r="B64" t="s">
+        <v>4059</v>
+      </c>
+      <c r="C64" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>4060</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4061</v>
+      </c>
+      <c r="C65" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>4062</v>
+      </c>
+      <c r="B66" t="s">
+        <v>4063</v>
+      </c>
+      <c r="C66" t="s">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>4064</v>
+      </c>
+      <c r="B67" t="s">
+        <v>4065</v>
+      </c>
+      <c r="C67" t="s">
         <v>3939</v>
       </c>
     </row>

</xml_diff>

<commit_message>
call things what they are: groups, group_time, baseline_reference, feature_type
</commit_message>
<xml_diff>
--- a/01_Processing/03_Quantification/c_data/quantification.xlsx
+++ b/01_Processing/03_Quantification/c_data/quantification.xlsx
@@ -155,10 +155,10 @@
     <t>Participant identifier.</t>
   </si>
   <si>
-    <t>group</t>
-  </si>
-  <si>
-    <t>Group the row belongs to (HR, LR, Hi, Lo, C1, C2), or a group cell such as HR_T1.</t>
+    <t>group_time</t>
+  </si>
+  <si>
+    <t>Group-by-time cell, such as HR_T1.</t>
   </si>
   <si>
     <t>blood_rel</t>
@@ -11822,7 +11822,7 @@
     <t>01_Processing/02_Normalisation/c_data/DAList_normalized.rds</t>
   </si>
   <si>
-    <t>39482f6e099d2d703c72e1364ec31471</t>
+    <t>ebdcad8bd54182d7e53ced5ad172b4ab</t>
   </si>
   <si>
     <t>BiocGenerics</t>

</xml_diff>